<commit_message>
Asset consolidation R2 + ship 3C iteration: prune 108 legacy assets, add Fab capital ships, GroundFire VFX, combat avatar, Mass notes
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeShip.xlsx
+++ b/data/Excel/GuLiStrikeShip.xlsx
@@ -3,170 +3,181 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="17680" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" windowHeight="17680" tabRatio="600" activeTab="1" autoFilterDateGrouping="true"/>
   </bookViews>
   <sheets>
-    <sheet name="Parts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tuning" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Parts" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="Tuning" sheetId="2" r:id="rId2" state="visible"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>Dreadnought</t>
+  </si>
+  <si>
+    <t>无畏舰 CombatAvatarFly-01 裸舰体；HullMeshOffset 为居中补偿(艏向+X)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="0"/>
   <fonts count="20">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <i val="1"/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="15"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color theme="0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -472,159 +483,159 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="false" pivotButton="false" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="false" pivotButton="false"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -677,7 +688,7 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -750,7 +761,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WPS">
   <a:themeElements>
     <a:clrScheme name="WPS">
       <a:dk1>
@@ -993,6 +1004,7 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1359,422 +1371,422 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="6"/>
   <cols>
-    <col width="10.9545454545455" customWidth="1" style="1" min="1" max="1"/>
-    <col width="11.6090909090909" customWidth="1" style="1" min="2" max="2"/>
-    <col width="13.8272727272727" customWidth="1" style="1" min="4" max="4"/>
-    <col width="14.5454545454545" customWidth="1" style="1" min="5" max="5"/>
-    <col width="18.8181818181818" customWidth="1" style="1" min="6" max="6"/>
-    <col width="22.2090909090909" customWidth="1" style="1" min="7" max="7"/>
-    <col width="21.2545454545455" customWidth="1" style="1" min="8" max="8"/>
-    <col width="20.3909090909091" customWidth="1" style="1" min="9" max="9"/>
-    <col width="25.6090909090909" customWidth="1" style="1" min="10" max="10"/>
-    <col width="18.5727272727273" customWidth="1" style="1" min="11" max="11"/>
-    <col width="15.1727272727273" customWidth="1" style="1" min="12" max="12"/>
-    <col width="18.4090909090909" customWidth="1" style="1" min="14" max="14"/>
-    <col width="15.9636363636364" customWidth="1" style="1" min="15" max="15"/>
-    <col width="15.8818181818182" customWidth="1" style="1" min="16" max="16"/>
-    <col width="17.4727272727273" customWidth="1" style="1" min="17" max="17"/>
-    <col width="16.8272727272727" customWidth="1" style="1" min="18" max="18"/>
-    <col width="17.7909090909091" customWidth="1" style="1" min="19" max="19"/>
-    <col width="21.3363636363636" customWidth="1" style="1" min="20" max="20"/>
-    <col width="17.6272727272727" customWidth="1" style="1" min="21" max="21"/>
-    <col width="18.5818181818182" customWidth="1" style="1" min="22" max="22"/>
-    <col width="19.7545454545455" customWidth="1" style="1" min="23" max="23"/>
-    <col width="17.9363636363636" customWidth="1" style="1" min="24" max="24"/>
-    <col width="16.9090909090909" customWidth="1" style="1" min="25" max="25"/>
+    <col customWidth="true" max="1" min="1" style="1" width="10.9545454545455"/>
+    <col customWidth="true" max="2" min="2" style="1" width="11.6090909090909"/>
+    <col customWidth="true" max="4" min="4" style="1" width="13.8272727272727"/>
+    <col customWidth="true" max="5" min="5" style="1" width="14.5454545454545"/>
+    <col customWidth="true" max="6" min="6" style="1" width="18.8181818181818"/>
+    <col customWidth="true" max="7" min="7" style="1" width="22.2090909090909"/>
+    <col customWidth="true" max="8" min="8" style="1" width="21.2545454545455"/>
+    <col customWidth="true" max="9" min="9" style="1" width="20.3909090909091"/>
+    <col customWidth="true" max="10" min="10" style="1" width="25.6090909090909"/>
+    <col customWidth="true" max="11" min="11" style="1" width="18.5727272727273"/>
+    <col customWidth="true" max="12" min="12" style="1" width="15.1727272727273"/>
+    <col customWidth="true" max="14" min="14" style="1" width="18.4090909090909"/>
+    <col customWidth="true" max="15" min="15" style="1" width="15.9636363636364"/>
+    <col customWidth="true" max="16" min="16" style="1" width="15.8818181818182"/>
+    <col customWidth="true" max="17" min="17" style="1" width="17.4727272727273"/>
+    <col customWidth="true" max="18" min="18" style="1" width="16.8272727272727"/>
+    <col customWidth="true" max="19" min="19" style="1" width="17.7909090909091"/>
+    <col customWidth="true" max="20" min="20" style="1" width="21.3363636363636"/>
+    <col customWidth="true" max="21" min="21" style="1" width="17.6272727272727"/>
+    <col customWidth="true" max="22" min="22" style="1" width="18.5818181818182"/>
+    <col customWidth="true" max="23" min="23" style="1" width="19.7545454545455"/>
+    <col customWidth="true" max="24" min="24" style="1" width="17.9363636363636"/>
+    <col customWidth="true" max="25" min="25" style="1" width="16.9090909090909"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="0" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="0" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="0" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="D1" s="0" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>HullMass</t>
         </is>
       </c>
-      <c r="E1" s="0" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>BaseMaxSpeed</t>
         </is>
       </c>
-      <c r="F1" s="0" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>BaseAcceleration</t>
         </is>
       </c>
-      <c r="G1" s="0" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>NominalThrustRatio</t>
         </is>
       </c>
-      <c r="H1" s="0" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>SpeedMultiplierMin</t>
         </is>
       </c>
-      <c r="I1" s="0" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SpeedMultiplierMax</t>
         </is>
       </c>
-      <c r="J1" s="0" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>BoostThrustMultiplier</t>
         </is>
       </c>
-      <c r="K1" s="0" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>MousePitchScale</t>
         </is>
       </c>
-      <c r="L1" s="0" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>MouseYawScale</t>
         </is>
       </c>
-      <c r="M1" s="0" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>YawRate</t>
         </is>
       </c>
-      <c r="N1" s="0" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>YawResponseSpeed</t>
         </is>
       </c>
-      <c r="O1" s="0" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>YawStopDamping</t>
         </is>
       </c>
-      <c r="P1" s="0" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>MaxBankAngle</t>
         </is>
       </c>
-      <c r="Q1" s="0" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>BankInterpSpeed</t>
         </is>
       </c>
-      <c r="R1" s="0" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>OrientTurnSpeed</t>
         </is>
       </c>
-      <c r="S1" s="0" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>OrientToMovement</t>
         </is>
       </c>
-      <c r="T1" s="0" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>OrientMinForwardDot</t>
         </is>
       </c>
-      <c r="U1" s="0" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>CameraPitchMin</t>
         </is>
       </c>
-      <c r="V1" s="0" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>CameraPitchMax</t>
         </is>
       </c>
-      <c r="W1" s="0" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>HullMeshOffsetX</t>
         </is>
       </c>
-      <c r="X1" s="0" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>HullMeshOffsetY</t>
         </is>
       </c>
-      <c r="Y1" s="0" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>HullMeshOffsetZ</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>str</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="H2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="I2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="J2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="K2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="L2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="M2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="N2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="O2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="P2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="Q2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="R2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="S2" s="0" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>bool</t>
         </is>
       </c>
-      <c r="T2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="U2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="V2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="W2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="X2" s="0" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="Y2" s="0" t="inlineStr">
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="D3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="H3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="I3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="K3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="L3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="M3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="N3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="O3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="P3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="Q3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="R3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="S3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="T3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="U3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="V3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="W3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="X3" s="0" t="inlineStr">
-        <is>
-          <t>Necessary</t>
-        </is>
-      </c>
-      <c r="Y3" s="0" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Necessary</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Necessary</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="n">
+      <c r="A4" t="n">
         <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1847,6 +1859,83 @@
       </c>
       <c r="Y4" t="n">
         <v>700</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1">
+        <v>100</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1200</v>
+      </c>
+      <c r="F5" s="1">
+        <v>400</v>
+      </c>
+      <c r="G5" s="1">
+        <v>6</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I5" s="1">
+        <v>2</v>
+      </c>
+      <c r="J5" s="1">
+        <v>2</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>40</v>
+      </c>
+      <c r="N5" s="1">
+        <v>3</v>
+      </c>
+      <c r="O5" s="1">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>4</v>
+      </c>
+      <c r="R5" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="S5" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="T5" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="U5" s="1">
+        <v>-80</v>
+      </c>
+      <c r="V5" s="1">
+        <v>80</v>
+      </c>
+      <c r="W5" s="1">
+        <v>-14162</v>
+      </c>
+      <c r="X5" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>-929</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: sync gameplay, weapon data, VFX, and authoring updates
Snapshot the accumulated GuLiStrike project changes through 2026-09-14,
including pooled 800 m/s wingman lasers, secondary weapon and spell-field
workbooks, resource gameplay, ship parts, unit feedback, map authoring,
art sources, documentation, and validation evidence.

Keep imported marketplace source packs, cooked acceptance builds, and
binary inspection backups local. Store authored art and visual evidence
with Git LFS without rewriting published history.

Validation: source-engine GuLiStrikeEditor and GuLiStrike Win64 Development
builds succeeded. Existing Wingman.Attack and CombatEffects checks passed
19 of 22; the three assertion failures are recorded in the project docs.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeShip.xlsx
+++ b/data/Excel/GuLiStrikeShip.xlsx
@@ -2,20 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <bookViews>
-    <workbookView activeTab="4"/>
+    <workbookView/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="1" r:id="Rf507666359b24463"/>
     <sheet name="Tuning" sheetId="2" r:id="R98cb5089503d4dc5"/>
     <sheet name="Camera" sheetId="3" r:id="Rb9ddd4ab1aae4aeb"/>
-    <sheet name="WingmanTargeting" sheetId="4" r:id="rId1"/>
-    <sheet name="WingmanWeapons" sheetId="5" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t xml:space="preserve">Dreadnought</t>
   </si>
@@ -216,6 +214,30 @@
   </si>
   <si>
     <t>AirDogfight</t>
+  </si>
+  <si>
+    <t>AirFireStartDistanceCentimeters</t>
+  </si>
+  <si>
+    <t>AirFireStopDistanceCentimeters</t>
+  </si>
+  <si>
+    <t>AirBurstDurationSeconds</t>
+  </si>
+  <si>
+    <t>AirOrbitCooldownSeconds</t>
+  </si>
+  <si>
+    <t>100m外开始5秒持续射击；50m内停止；返舰盘旋冷却3秒</t>
+  </si>
+  <si>
+    <t>AirBurstOrbit</t>
+  </si>
+  <si>
+    <t>EffectConfigId</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -1879,10 +1901,10 @@
         <v>100</v>
       </c>
       <c r="E5" s="1">
-        <v>5400</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>600</v>
+        <v>16200</v>
+      </c>
+      <c r="F5" s="1">
+        <v>2400</v>
       </c>
       <c r="G5" s="1">
         <v>6</v>
@@ -1903,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="M5">
-        <v>40</v>
+        <v>13.333333</v>
       </c>
       <c r="N5" s="1">
         <v>3</v>
@@ -2123,602 +2145,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" t="s">
-        <v>53</v>
-      </c>
-      <c r="G1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4">
-        <v>150000</v>
-      </c>
-      <c r="E4">
-        <v>180000</v>
-      </c>
-      <c r="F4">
-        <v>0.8</v>
-      </c>
-      <c r="G4">
-        <v>0.2</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N1" t="s">
-        <v>32</v>
-      </c>
-      <c r="O1" t="s">
-        <v>33</v>
-      </c>
-      <c r="P1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>55</v>
-      </c>
-      <c r="R1" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" t="s">
-        <v>57</v>
-      </c>
-      <c r="T1" t="s">
-        <v>58</v>
-      </c>
-      <c r="U1" t="s">
-        <v>59</v>
-      </c>
-      <c r="V1" t="s">
-        <v>60</v>
-      </c>
-      <c r="W1" t="s">
-        <v>61</v>
-      </c>
-      <c r="X1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>64</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N2" t="s">
-        <v>15</v>
-      </c>
-      <c r="O2" t="s">
-        <v>15</v>
-      </c>
-      <c r="P2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>15</v>
-      </c>
-      <c r="R2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" t="s">
-        <v>15</v>
-      </c>
-      <c r="T2" t="s">
-        <v>15</v>
-      </c>
-      <c r="U2" t="s">
-        <v>15</v>
-      </c>
-      <c r="V2" t="s">
-        <v>15</v>
-      </c>
-      <c r="W2" t="s">
-        <v>15</v>
-      </c>
-      <c r="X2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M3" t="s">
-        <v>16</v>
-      </c>
-      <c r="N3" t="s">
-        <v>16</v>
-      </c>
-      <c r="O3" t="s">
-        <v>16</v>
-      </c>
-      <c r="P3" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>16</v>
-      </c>
-      <c r="R3" t="s">
-        <v>16</v>
-      </c>
-      <c r="S3" t="s">
-        <v>16</v>
-      </c>
-      <c r="T3" t="s">
-        <v>16</v>
-      </c>
-      <c r="U3" t="s">
-        <v>16</v>
-      </c>
-      <c r="V3" t="s">
-        <v>16</v>
-      </c>
-      <c r="W3" t="s">
-        <v>16</v>
-      </c>
-      <c r="X3" t="s">
-        <v>16</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>16</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G4">
-        <v>10</v>
-      </c>
-      <c r="H4">
-        <v>0.5</v>
-      </c>
-      <c r="I4">
-        <v>150000</v>
-      </c>
-      <c r="J4">
-        <v>20</v>
-      </c>
-      <c r="K4">
-        <v>4500</v>
-      </c>
-      <c r="L4">
-        <v>1.5</v>
-      </c>
-      <c r="M4">
-        <v>10</v>
-      </c>
-      <c r="N4">
-        <v>12000</v>
-      </c>
-      <c r="O4">
-        <v>10000</v>
-      </c>
-      <c r="P4">
-        <v>800</v>
-      </c>
-      <c r="Q4">
-        <v>30000</v>
-      </c>
-      <c r="R4">
-        <v>45000</v>
-      </c>
-      <c r="S4">
-        <v>0.35</v>
-      </c>
-      <c r="T4">
-        <v>0.6</v>
-      </c>
-      <c r="U4">
-        <v>15000</v>
-      </c>
-      <c r="V4">
-        <v>10000</v>
-      </c>
-      <c r="W4">
-        <v>7500</v>
-      </c>
-      <c r="X4">
-        <v>40</v>
-      </c>
-      <c r="Y4">
-        <v>90</v>
-      </c>
-      <c r="Z4">
-        <v>30</v>
-      </c>
-      <c r="AA4">
-        <v>120000</v>
-      </c>
-      <c r="AB4">
-        <v>1.5</v>
-      </c>
-      <c r="AC4">
-        <v>45</v>
-      </c>
-      <c r="AD4">
-        <v>1200</v>
-      </c>
-      <c r="AE4">
-        <v>0</v>
-      </c>
-      <c r="AF4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5">
-        <v>30</v>
-      </c>
-      <c r="H5">
-        <v>8</v>
-      </c>
-      <c r="I5">
-        <v>150000</v>
-      </c>
-      <c r="J5">
-        <v>20</v>
-      </c>
-      <c r="K5">
-        <v>4500</v>
-      </c>
-      <c r="L5">
-        <v>1.5</v>
-      </c>
-      <c r="M5">
-        <v>10</v>
-      </c>
-      <c r="N5">
-        <v>12000</v>
-      </c>
-      <c r="O5">
-        <v>10000</v>
-      </c>
-      <c r="P5">
-        <v>800</v>
-      </c>
-      <c r="Q5">
-        <v>30000</v>
-      </c>
-      <c r="R5">
-        <v>45000</v>
-      </c>
-      <c r="S5">
-        <v>0.35</v>
-      </c>
-      <c r="T5">
-        <v>0.6</v>
-      </c>
-      <c r="U5">
-        <v>15000</v>
-      </c>
-      <c r="V5">
-        <v>10000</v>
-      </c>
-      <c r="W5">
-        <v>7500</v>
-      </c>
-      <c r="X5">
-        <v>40</v>
-      </c>
-      <c r="Y5">
-        <v>90</v>
-      </c>
-      <c r="Z5">
-        <v>30</v>
-      </c>
-      <c r="AA5">
-        <v>6000</v>
-      </c>
-      <c r="AB5">
-        <v>8</v>
-      </c>
-      <c r="AC5">
-        <v>30</v>
-      </c>
-      <c r="AD5">
-        <v>1200</v>
-      </c>
-      <c r="AE5">
-        <v>0</v>
-      </c>
-      <c r="AF5">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: retire legacy projectiles and resolve PIE crowd capacity crash
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeShip.xlsx
+++ b/data/Excel/GuLiStrikeShip.xlsx
@@ -1359,7 +1359,6 @@
     <col customWidth="true" max="4" min="4" style="1" width="17.863636016845703"/>
     <col customWidth="true" max="5" min="5" style="1" width="10.172727584838867"/>
     <col customWidth="true" max="6" min="6" style="1" width="12.363636016845703"/>
-    <col customWidth="true" max="13" min="13" style="1" width="66.59091186523438"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1385,24 +1384,15 @@
         <v>79</v>
       </c>
       <c r="H1" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I1" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="J1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="N1" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1438,15 +1428,6 @@
         <v>15</v>
       </c>
       <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N2" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1482,15 +1463,6 @@
         <v>17</v>
       </c>
       <c r="K3" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" t="s">
-        <v>17</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="N3" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1525,16 +1497,7 @@
       <c r="J4" t="s">
         <v>74</v>
       </c>
-      <c r="K4" t="s">
-        <v>74</v>
-      </c>
-      <c r="L4" t="s">
-        <v>74</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="N4">
+      <c r="K4">
         <v>5901</v>
       </c>
     </row>
@@ -1569,16 +1532,7 @@
       <c r="J5" t="s">
         <v>74</v>
       </c>
-      <c r="K5" t="s">
-        <v>74</v>
-      </c>
-      <c r="L5" t="s">
-        <v>74</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="N5">
+      <c r="K5">
         <v>5902</v>
       </c>
     </row>
@@ -1605,24 +1559,15 @@
         <v>74</v>
       </c>
       <c r="H6">
-        <v>10</v>
+        <v>350</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N6">
         <v>5903</v>
       </c>
     </row>
@@ -1649,24 +1594,15 @@
         <v>74</v>
       </c>
       <c r="H7">
-        <v>40</v>
+        <v>450</v>
       </c>
       <c r="I7">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N7">
         <v>5904</v>
       </c>
     </row>
@@ -1693,24 +1629,15 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N8">
         <v>5101</v>
       </c>
     </row>
@@ -1737,24 +1664,15 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N9">
         <v>5102</v>
       </c>
     </row>
@@ -1781,24 +1699,15 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N10">
         <v>5103</v>
       </c>
     </row>
@@ -1825,24 +1734,15 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N11">
         <v>5104</v>
       </c>
     </row>
@@ -1869,24 +1769,15 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N12">
         <v>5105</v>
       </c>
     </row>
@@ -1913,24 +1804,15 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N13">
         <v>5106</v>
       </c>
     </row>
@@ -1957,24 +1839,15 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N14">
         <v>5107</v>
       </c>
     </row>
@@ -2010,15 +1883,6 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="N15">
         <v>5108</v>
       </c>
     </row>
@@ -2054,15 +1918,6 @@
         <v>0</v>
       </c>
       <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="N16">
         <v>5109</v>
       </c>
     </row>
@@ -2089,24 +1944,15 @@
         <v>0</v>
       </c>
       <c r="H17">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N17">
         <v>5110</v>
       </c>
     </row>
@@ -2133,24 +1979,15 @@
         <v>0</v>
       </c>
       <c r="H18">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N18">
         <v>5111</v>
       </c>
     </row>
@@ -2186,15 +2023,6 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="N19">
         <v>5112</v>
       </c>
     </row>
@@ -2221,24 +2049,15 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N20">
         <v>5113</v>
       </c>
     </row>
@@ -2265,24 +2084,15 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N21">
         <v>5113</v>
       </c>
     </row>

</xml_diff>